<commit_message>
Update figures, tables and scripts - final pre-submission
Figures:
- Updated Fig1-4 main figures
- Updated FigS1-S3 supplementary figures
- Renamed FigS4→FigS5 regression residuals (new numbering)
- Removed old FigS4

Scripts R:
- Renamed figS2-S5 to figS1-S4 (matching new figure numbering)
- Updated fig1-4 with final corrections
- Updated 10_temporal_dynamics.R

Tables:
- TableS1-S5 XLSX updated
- TableS9 CSV+XLSX: added primary PERMANOVA row (R2=0.106, F=424.0)
- TableS8: restored ACICU reference genome (20,739 total)
</commit_message>
<xml_diff>
--- a/results/supplementary/tables_submission/TableS3_temporal_trends_FDR.xlsx
+++ b/results/supplementary/tables_submission/TableS3_temporal_trends_FDR.xlsx
@@ -25,25 +25,25 @@
     <t xml:space="preserve">Gene</t>
   </si>
   <si>
-    <t xml:space="preserve">Resistance_class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slope_per_year</t>
+    <t xml:space="preserve">Resistance class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slope per year</t>
   </si>
   <si>
     <t xml:space="preserve">R2</t>
   </si>
   <si>
-    <t xml:space="preserve">P_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q_value_BH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sig_p005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sig_q005</t>
+    <t xml:space="preserve">P value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q value BH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sig p005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sig q005</t>
   </si>
   <si>
     <t xml:space="preserve">Trend</t>
@@ -360,28 +360,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -640,1314 +644,1314 @@
   <dimension ref="A1:I42"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="14.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="14.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>0.025379</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>0.576</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G2" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H2" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="s">
+      <c r="G2" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>0.024633</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>0.6331</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G3" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H3" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I3" s="4" t="s">
+      <c r="G3" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H3" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>0.022347</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>0.8299</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G4" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H4" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="G4" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>-0.018653</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.8303</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G5" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H5" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I5" s="4" t="s">
+      <c r="G5" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H5" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>-0.015292</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>0.6001</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G6" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H6" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I6" s="2" t="s">
+      <c r="G6" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>-0.016769</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>0.633</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G7" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I7" s="4" t="s">
+      <c r="G7" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="3" t="n">
         <v>-0.013278</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>0.667</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G8" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H8" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="s">
+      <c r="G8" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>-0.013972</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>0.817</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G9" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H9" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I9" s="4" t="s">
+      <c r="G9" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H9" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="3" t="n">
         <v>0.004102</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="3" t="n">
         <v>0.7623</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G10" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H10" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I10" s="2" t="s">
+      <c r="G10" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="5" t="n">
         <v>0.024578</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>0.5525</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.00041</v>
       </c>
-      <c r="G11" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H11" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I11" s="4" t="s">
+      <c r="G11" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H11" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="3" t="n">
         <v>-0.004792</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="3" t="n">
         <v>0.4948</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="3" t="n">
         <v>0.001025</v>
       </c>
-      <c r="G12" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H12" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I12" s="2" t="s">
+      <c r="G12" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I12" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>-0.004735</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>0.4917</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="5" t="n">
         <v>0.001025</v>
       </c>
-      <c r="G13" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H13" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I13" s="4" t="s">
+      <c r="G13" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H13" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I13" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="3" t="n">
         <v>0.018513</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <v>0.4324</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>0.0009</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="3" t="n">
         <v>0.002838</v>
       </c>
-      <c r="G14" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H14" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="G14" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="5" t="n">
         <v>-0.007614</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>0.3741</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="5" t="n">
         <v>0.0025</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="5" t="n">
         <v>0.007321</v>
       </c>
-      <c r="G15" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H15" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I15" s="4" t="s">
+      <c r="G15" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H15" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I15" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="3" t="n">
         <v>-0.010949</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="3" t="n">
         <v>0.3684</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>0.0027</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="3" t="n">
         <v>0.00738</v>
       </c>
-      <c r="G16" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H16" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="G16" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H16" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="5" t="n">
         <v>0.001419</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>0.2799</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="5" t="n">
         <v>0.0113</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" s="5" t="n">
         <v>0.028941</v>
       </c>
-      <c r="G17" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H17" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I17" s="4" t="s">
+      <c r="G17" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H17" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I17" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="3" t="n">
         <v>-0.003377</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="3" t="n">
         <v>0.2765</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="3" t="n">
         <v>0.012</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="3" t="n">
         <v>0.028941</v>
       </c>
-      <c r="G18" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H18" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="G18" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H18" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="5" t="n">
         <v>-0.007687</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>0.2393</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>0.0209</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="F19" s="5" t="n">
         <v>0.047606</v>
       </c>
-      <c r="G19" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H19" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I19" s="4" t="s">
+      <c r="G19" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H19" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="I19" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="3" t="n">
         <v>0.001347</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="3" t="n">
         <v>0.2188</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="3" t="n">
         <v>0.0281</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="3" t="n">
         <v>0.060637</v>
       </c>
-      <c r="G20" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H20" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="2" t="s">
+      <c r="G20" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H20" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="5" t="n">
         <v>0.005835</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="5" t="n">
         <v>0.2133</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="5" t="n">
         <v>0.0305</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F21" s="5" t="n">
         <v>0.062525</v>
       </c>
-      <c r="G21" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H21" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I21" s="4" t="s">
+      <c r="G21" s="6" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C22" s="3" t="n">
         <v>0.003631</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="3" t="n">
         <v>0.1799</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="3" t="n">
         <v>0.0491</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="3" t="n">
         <v>0.095862</v>
       </c>
-      <c r="G22" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H22" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I22" s="2" t="s">
+      <c r="G22" s="4" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H22" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="5" t="n">
         <v>0.004947</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="5" t="n">
         <v>0.1526</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="5" t="n">
         <v>0.0723</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" s="5" t="n">
         <v>0.134741</v>
       </c>
-      <c r="G23" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I23" s="4" t="s">
+      <c r="G23" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C24" s="3" t="n">
         <v>0.005817</v>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="3" t="n">
         <v>0.1448</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="3" t="n">
         <v>0.0807</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="3" t="n">
         <v>0.143856</v>
       </c>
-      <c r="G24" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="2" t="s">
+      <c r="G24" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="5" t="n">
         <v>0.000832</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" s="5" t="n">
         <v>0.1172</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="5" t="n">
         <v>0.1189</v>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="F25" s="5" t="n">
         <v>0.203121</v>
       </c>
-      <c r="G25" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H25" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I25" s="4" t="s">
+      <c r="G25" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C26" s="3" t="n">
         <v>0.000119</v>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="3" t="n">
         <v>0.1023</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="3" t="n">
         <v>0.1468</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="3" t="n">
         <v>0.240752</v>
       </c>
-      <c r="G26" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="2" t="s">
+      <c r="G26" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="5" t="n">
         <v>0.005719</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D27" s="5" t="n">
         <v>0.0834</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="5" t="n">
         <v>0.1923</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="F27" s="5" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G27" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I27" s="4" t="s">
+      <c r="G27" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C28" s="3" t="n">
         <v>0.000151</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D28" s="3" t="n">
         <v>0.0823</v>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="E28" s="3" t="n">
         <v>0.1955</v>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="F28" s="3" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G28" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I28" s="2" t="s">
+      <c r="G28" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="5" t="n">
         <v>0.003316</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" s="5" t="n">
         <v>0.0787</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="5" t="n">
         <v>0.206</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="F29" s="5" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G29" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I29" s="4" t="s">
+      <c r="G29" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C30" s="3" t="n">
         <v>2.6E-005</v>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="D30" s="3" t="n">
         <v>0.0787</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="3" t="n">
         <v>0.2061</v>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="3" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G30" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H30" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I30" s="2" t="s">
+      <c r="G30" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="5" t="n">
         <v>0.000141</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" s="5" t="n">
         <v>0.0752</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" s="5" t="n">
         <v>0.2167</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="F31" s="5" t="n">
         <v>0.296157</v>
       </c>
-      <c r="G31" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H31" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I31" s="4" t="s">
+      <c r="G31" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C32" s="3" t="n">
         <v>0.000153</v>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D32" s="3" t="n">
         <v>0.0574</v>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E32" s="3" t="n">
         <v>0.283</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="3" t="n">
         <v>0.37429</v>
       </c>
-      <c r="G32" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="2" t="s">
+      <c r="G32" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="5" t="n">
         <v>0.003998</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="5" t="n">
         <v>0.0484</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" s="5" t="n">
         <v>0.3254</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="F33" s="5" t="n">
         <v>0.416919</v>
       </c>
-      <c r="G33" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H33" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I33" s="4" t="s">
+      <c r="G33" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C34" s="3" t="n">
         <v>-0.002778</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D34" s="3" t="n">
         <v>0.0427</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E34" s="3" t="n">
         <v>0.3561</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="3" t="n">
         <v>0.442427</v>
       </c>
-      <c r="G34" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H34" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I34" s="2" t="s">
+      <c r="G34" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="5" t="n">
         <v>-2.8E-005</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D35" s="5" t="n">
         <v>0.0082</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E35" s="5" t="n">
         <v>0.6885</v>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="F35" s="5" t="n">
         <v>0.824217</v>
       </c>
-      <c r="G35" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H35" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="4" t="s">
+      <c r="G35" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C36" s="3" t="n">
         <v>2E-006</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="3" t="n">
         <v>0.0074</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E36" s="3" t="n">
         <v>0.7036</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="3" t="n">
         <v>0.824217</v>
       </c>
-      <c r="G36" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H36" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I36" s="2" t="s">
+      <c r="G36" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="5" t="n">
         <v>-0.000139</v>
       </c>
-      <c r="D37" s="4" t="n">
+      <c r="D37" s="5" t="n">
         <v>0.006</v>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" s="5" t="n">
         <v>0.7319</v>
       </c>
-      <c r="F37" s="4" t="n">
+      <c r="F37" s="5" t="n">
         <v>0.833553</v>
       </c>
-      <c r="G37" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H37" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="4" t="s">
+      <c r="G37" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="2" t="n">
+      <c r="C38" s="3" t="n">
         <v>0.000246</v>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="3" t="n">
         <v>0.0048</v>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="3" t="n">
         <v>0.7591</v>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="F38" s="3" t="n">
         <v>0.841165</v>
       </c>
-      <c r="G38" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H38" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I38" s="2" t="s">
+      <c r="G38" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="5" t="n">
         <v>-0.000231</v>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="5" t="n">
         <v>0.0016</v>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="5" t="n">
         <v>0.8597</v>
       </c>
-      <c r="F39" s="4" t="n">
+      <c r="F39" s="5" t="n">
         <v>0.908308</v>
       </c>
-      <c r="G39" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I39" s="4" t="s">
+      <c r="G39" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C40" s="3" t="n">
         <v>2.2E-005</v>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="3" t="n">
         <v>0.0015</v>
       </c>
-      <c r="E40" s="2" t="n">
+      <c r="E40" s="3" t="n">
         <v>0.864</v>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="F40" s="3" t="n">
         <v>0.908308</v>
       </c>
-      <c r="G40" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H40" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I40" s="2" t="s">
+      <c r="G40" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="5" t="n">
         <v>-4E-006</v>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D41" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" s="5" t="n">
         <v>0.9406</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="F41" s="5" t="n">
         <v>0.964115</v>
       </c>
-      <c r="G41" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H41" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I41" s="4" t="s">
+      <c r="G41" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H42" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I42" s="2" t="s">
+      <c r="C42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I42" s="3" t="s">
         <v>78</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update figures, scripts and TableS3 - final corrections
Figures:
- Updated Fig1, Fig2, Fig3 (visual corrections)
- Renamed FigS5_regression_residuals → FigS4_regression_residuals

Scripts R:
- Updated fig1_network_v1.R, fig2_heatmap_v1.R, fig3_onehealth_v1.R

Tables:
- Updated TableS3_temporal_trends_FDR (CSV + XLSX)
</commit_message>
<xml_diff>
--- a/results/supplementary/tables_submission/TableS3_temporal_trends_FDR.xlsx
+++ b/results/supplementary/tables_submission/TableS3_temporal_trends_FDR.xlsx
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Trend</t>
   </si>
   <si>
-    <t xml:space="preserve">msr(e)</t>
+    <t xml:space="preserve">msr(E)</t>
   </si>
   <si>
     <t xml:space="preserve">Macrolide</t>
@@ -58,13 +58,13 @@
     <t xml:space="preserve">increasing</t>
   </si>
   <si>
-    <t xml:space="preserve">arma</t>
+    <t xml:space="preserve">armA</t>
   </si>
   <si>
     <t xml:space="preserve">Aminoglycoside (16S methylase)</t>
   </si>
   <si>
-    <t xml:space="preserve">ftsi</t>
+    <t xml:space="preserve">ftsI</t>
   </si>
   <si>
     <t xml:space="preserve">Beta-lactam (PBP3)</t>
@@ -79,7 +79,7 @@
     <t xml:space="preserve">decreasing</t>
   </si>
   <si>
-    <t xml:space="preserve">qacedelta</t>
+    <t xml:space="preserve">qacEΔ1</t>
   </si>
   <si>
     <t xml:space="preserve">Disinfectant (QAC)</t>
@@ -97,37 +97,37 @@
     <t xml:space="preserve">Sulfonamide</t>
   </si>
   <si>
-    <t xml:space="preserve">blandm</t>
+    <t xml:space="preserve">blaNDM</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem (MBL)</t>
   </si>
   <si>
-    <t xml:space="preserve">mph(e)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mert</t>
+    <t xml:space="preserve">mph(E)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">merT</t>
   </si>
   <si>
     <t xml:space="preserve">Metal resistance</t>
   </si>
   <si>
-    <t xml:space="preserve">merr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blaoxa_23like</t>
+    <t xml:space="preserve">merR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blaOXA-23-like</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem (OXA-23)</t>
   </si>
   <si>
-    <t xml:space="preserve">blatem</t>
+    <t xml:space="preserve">blaTEM</t>
   </si>
   <si>
     <t xml:space="preserve">Beta-lactam (TEM)</t>
   </si>
   <si>
-    <t xml:space="preserve">aada</t>
+    <t xml:space="preserve">aadA</t>
   </si>
   <si>
     <t xml:space="preserve">arr-2</t>
@@ -136,31 +136,31 @@
     <t xml:space="preserve">Rifampicin</t>
   </si>
   <si>
-    <t xml:space="preserve">blaoxa_58like</t>
+    <t xml:space="preserve">blaOXA-58-like</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem (OXA-58)</t>
   </si>
   <si>
-    <t xml:space="preserve">adec</t>
+    <t xml:space="preserve">adeC</t>
   </si>
   <si>
     <t xml:space="preserve">Efflux pump (AdeABC)</t>
   </si>
   <si>
-    <t xml:space="preserve">pmrb</t>
+    <t xml:space="preserve">pmrB</t>
   </si>
   <si>
     <t xml:space="preserve">Colistin (pmrB)</t>
   </si>
   <si>
-    <t xml:space="preserve">tet(b)</t>
+    <t xml:space="preserve">tet(B)</t>
   </si>
   <si>
     <t xml:space="preserve">Tetracycline</t>
   </si>
   <si>
-    <t xml:space="preserve">blaoxa_24like</t>
+    <t xml:space="preserve">blaOXA-24-like</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem (OXA-24)</t>
@@ -169,19 +169,19 @@
     <t xml:space="preserve">aph(3'')</t>
   </si>
   <si>
-    <t xml:space="preserve">parc</t>
+    <t xml:space="preserve">parC</t>
   </si>
   <si>
     <t xml:space="preserve">Quinolone (QRDR)</t>
   </si>
   <si>
-    <t xml:space="preserve">blaoxa_235like</t>
+    <t xml:space="preserve">blaOXA-235-like</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem (OXA-235)</t>
   </si>
   <si>
-    <t xml:space="preserve">tet(x5)</t>
+    <t xml:space="preserve">tet(X5)</t>
   </si>
   <si>
     <t xml:space="preserve">Tetracycline (Tet-X5)</t>
@@ -196,10 +196,10 @@
     <t xml:space="preserve">aph(6)</t>
   </si>
   <si>
-    <t xml:space="preserve">blavim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tet(x3)</t>
+    <t xml:space="preserve">blaVIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tet(X3)</t>
   </si>
   <si>
     <t xml:space="preserve">Tetracycline (Tet-X3)</t>
@@ -211,16 +211,16 @@
     <t xml:space="preserve">Colistin</t>
   </si>
   <si>
-    <t xml:space="preserve">catb</t>
+    <t xml:space="preserve">catB</t>
   </si>
   <si>
     <t xml:space="preserve">Phenicol</t>
   </si>
   <si>
-    <t xml:space="preserve">gyra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blakpc</t>
+    <t xml:space="preserve">gyrA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blaKPC</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem</t>
@@ -229,28 +229,28 @@
     <t xml:space="preserve">arr</t>
   </si>
   <si>
-    <t xml:space="preserve">blaoxa_143like</t>
+    <t xml:space="preserve">BlaOXA-143-like</t>
   </si>
   <si>
     <t xml:space="preserve">Carbapenem (OXA-143)</t>
   </si>
   <si>
-    <t xml:space="preserve">abaf</t>
+    <t xml:space="preserve">abaF</t>
   </si>
   <si>
     <t xml:space="preserve">Fosfomycin</t>
   </si>
   <si>
-    <t xml:space="preserve">dfra</t>
+    <t xml:space="preserve">dfrA</t>
   </si>
   <si>
     <t xml:space="preserve">Trimethoprim</t>
   </si>
   <si>
-    <t xml:space="preserve">rpob</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blaimp</t>
+    <t xml:space="preserve">rpoB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blaIMP</t>
   </si>
   <si>
     <t xml:space="preserve">mcr-4.7</t>
@@ -647,10 +647,12 @@
       <c r="F2" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G2" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="6" t="b">
+      <c r="G2" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I2" s="4" t="s">
@@ -676,10 +678,12 @@
       <c r="F3" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G3" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="6" t="b">
+      <c r="G3" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="4" t="s">
@@ -705,10 +709,12 @@
       <c r="F4" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G4" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6" t="b">
+      <c r="G4" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I4" s="4" t="s">
@@ -734,10 +740,12 @@
       <c r="F5" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G5" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="6" t="b">
+      <c r="G5" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
@@ -763,10 +771,12 @@
       <c r="F6" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G6" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="6" t="b">
+      <c r="G6" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I6" s="4" t="s">
@@ -792,10 +802,12 @@
       <c r="F7" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G7" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="6" t="b">
+      <c r="G7" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I7" s="4" t="s">
@@ -821,10 +833,12 @@
       <c r="F8" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G8" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="6" t="b">
+      <c r="G8" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I8" s="4" t="s">
@@ -850,10 +864,12 @@
       <c r="F9" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G9" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="6" t="b">
+      <c r="G9" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I9" s="4" t="s">
@@ -879,10 +895,12 @@
       <c r="F10" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="G10" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="6" t="b">
+      <c r="G10" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I10" s="4" t="s">
@@ -908,10 +926,12 @@
       <c r="F11" s="5" t="n">
         <v>0.00041</v>
       </c>
-      <c r="G11" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="6" t="b">
+      <c r="G11" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I11" s="4" t="s">
@@ -937,10 +957,12 @@
       <c r="F12" s="5" t="n">
         <v>0.001025</v>
       </c>
-      <c r="G12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="6" t="b">
+      <c r="G12" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I12" s="4" t="s">
@@ -966,10 +988,12 @@
       <c r="F13" s="5" t="n">
         <v>0.001025</v>
       </c>
-      <c r="G13" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="6" t="b">
+      <c r="G13" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I13" s="4" t="s">
@@ -995,10 +1019,12 @@
       <c r="F14" s="5" t="n">
         <v>0.002838</v>
       </c>
-      <c r="G14" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" s="6" t="b">
+      <c r="G14" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I14" s="4" t="s">
@@ -1024,10 +1050,12 @@
       <c r="F15" s="5" t="n">
         <v>0.007321</v>
       </c>
-      <c r="G15" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" s="6" t="b">
+      <c r="G15" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I15" s="4" t="s">
@@ -1053,10 +1081,12 @@
       <c r="F16" s="5" t="n">
         <v>0.00738</v>
       </c>
-      <c r="G16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" s="6" t="b">
+      <c r="G16" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I16" s="4" t="s">
@@ -1082,10 +1112,12 @@
       <c r="F17" s="5" t="n">
         <v>0.028941</v>
       </c>
-      <c r="G17" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" s="6" t="b">
+      <c r="G17" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I17" s="4" t="s">
@@ -1111,10 +1143,12 @@
       <c r="F18" s="5" t="n">
         <v>0.028941</v>
       </c>
-      <c r="G18" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" s="6" t="b">
+      <c r="G18" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I18" s="4" t="s">
@@ -1140,10 +1174,12 @@
       <c r="F19" s="5" t="n">
         <v>0.047606</v>
       </c>
-      <c r="G19" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="6" t="b">
+      <c r="G19" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I19" s="4" t="s">
@@ -1169,10 +1205,12 @@
       <c r="F20" s="5" t="n">
         <v>0.060637</v>
       </c>
-      <c r="G20" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" s="6" t="b">
+      <c r="G20" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I20" s="4" t="s">
@@ -1198,10 +1236,12 @@
       <c r="F21" s="5" t="n">
         <v>0.062525</v>
       </c>
-      <c r="G21" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" s="6" t="b">
+      <c r="G21" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I21" s="4" t="s">
@@ -1227,10 +1267,12 @@
       <c r="F22" s="5" t="n">
         <v>0.095862</v>
       </c>
-      <c r="G22" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="6" t="b">
+      <c r="G22" s="6" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I22" s="4" t="s">
@@ -1256,10 +1298,12 @@
       <c r="F23" s="5" t="n">
         <v>0.134741</v>
       </c>
-      <c r="G23" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H23" s="6" t="b">
+      <c r="G23" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I23" s="4" t="s">
@@ -1285,10 +1329,12 @@
       <c r="F24" s="5" t="n">
         <v>0.143856</v>
       </c>
-      <c r="G24" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24" s="6" t="b">
+      <c r="G24" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I24" s="4" t="s">
@@ -1314,10 +1360,12 @@
       <c r="F25" s="5" t="n">
         <v>0.203121</v>
       </c>
-      <c r="G25" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H25" s="6" t="b">
+      <c r="G25" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I25" s="4" t="s">
@@ -1343,10 +1391,12 @@
       <c r="F26" s="5" t="n">
         <v>0.240752</v>
       </c>
-      <c r="G26" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H26" s="6" t="b">
+      <c r="G26" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I26" s="4" t="s">
@@ -1372,10 +1422,12 @@
       <c r="F27" s="5" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G27" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H27" s="6" t="b">
+      <c r="G27" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I27" s="4" t="s">
@@ -1401,10 +1453,12 @@
       <c r="F28" s="5" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G28" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" s="6" t="b">
+      <c r="G28" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I28" s="4" t="s">
@@ -1430,10 +1484,12 @@
       <c r="F29" s="5" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G29" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H29" s="6" t="b">
+      <c r="G29" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I29" s="4" t="s">
@@ -1459,10 +1515,12 @@
       <c r="F30" s="5" t="n">
         <v>0.291383</v>
       </c>
-      <c r="G30" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H30" s="6" t="b">
+      <c r="G30" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I30" s="4" t="s">
@@ -1488,10 +1546,12 @@
       <c r="F31" s="5" t="n">
         <v>0.296157</v>
       </c>
-      <c r="G31" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H31" s="6" t="b">
+      <c r="G31" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I31" s="4" t="s">
@@ -1517,10 +1577,12 @@
       <c r="F32" s="5" t="n">
         <v>0.37429</v>
       </c>
-      <c r="G32" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H32" s="6" t="b">
+      <c r="G32" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I32" s="4" t="s">
@@ -1546,10 +1608,12 @@
       <c r="F33" s="5" t="n">
         <v>0.416919</v>
       </c>
-      <c r="G33" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H33" s="6" t="b">
+      <c r="G33" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I33" s="4" t="s">
@@ -1575,10 +1639,12 @@
       <c r="F34" s="5" t="n">
         <v>0.442427</v>
       </c>
-      <c r="G34" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H34" s="6" t="b">
+      <c r="G34" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I34" s="4" t="s">
@@ -1604,10 +1670,12 @@
       <c r="F35" s="5" t="n">
         <v>0.824217</v>
       </c>
-      <c r="G35" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H35" s="6" t="b">
+      <c r="G35" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I35" s="4" t="s">
@@ -1633,10 +1701,12 @@
       <c r="F36" s="5" t="n">
         <v>0.824217</v>
       </c>
-      <c r="G36" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H36" s="6" t="b">
+      <c r="G36" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I36" s="4" t="s">
@@ -1662,10 +1732,12 @@
       <c r="F37" s="5" t="n">
         <v>0.833553</v>
       </c>
-      <c r="G37" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H37" s="6" t="b">
+      <c r="G37" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I37" s="4" t="s">
@@ -1691,10 +1763,12 @@
       <c r="F38" s="5" t="n">
         <v>0.841165</v>
       </c>
-      <c r="G38" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H38" s="6" t="b">
+      <c r="G38" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I38" s="4" t="s">
@@ -1720,10 +1794,12 @@
       <c r="F39" s="5" t="n">
         <v>0.908308</v>
       </c>
-      <c r="G39" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H39" s="6" t="b">
+      <c r="G39" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I39" s="4" t="s">
@@ -1749,10 +1825,12 @@
       <c r="F40" s="5" t="n">
         <v>0.908308</v>
       </c>
-      <c r="G40" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H40" s="6" t="b">
+      <c r="G40" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I40" s="4" t="s">
@@ -1778,10 +1856,12 @@
       <c r="F41" s="5" t="n">
         <v>0.964115</v>
       </c>
-      <c r="G41" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H41" s="6" t="b">
+      <c r="G41" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I41" s="4" t="s">
@@ -1807,10 +1887,12 @@
       <c r="F42" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H42" s="6" t="b">
+      <c r="G42" s="6" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="I42" s="4" t="s">

</xml_diff>